<commit_message>
Bâtiment 30x10 : en-tête et identité Asseya Silver Construction sur tous les documents
Logo, coordonnées, N° CC, RCCM, banque et régime fiscal repris du devis ASC
du 16/02/2026 ; zone cachet/signature entreprise ; auteur Moulo Jean Claude.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y2qTq9Y3zXHLMLHGTW5fBh
</commit_message>
<xml_diff>
--- a/docs/projets/batiment-industriel-30x10/Batiment_30x10_Metre_DS_DQE.xlsx
+++ b/docs/projets/batiment-industriel-30x10/Batiment_30x10_Metre_DS_DQE.xlsx
@@ -207,7 +207,7 @@
     <numFmt numFmtId="169" formatCode="0.000"/>
     <numFmt numFmtId="170" formatCode="#,##0.000;(#,##0.000);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -251,6 +251,11 @@
       <name val="Arial"/>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="7">
@@ -356,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -408,6 +413,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,6 +488,66 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="904875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -773,323 +839,420 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Notice du classeur - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Notice du classeur - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Objet</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Métré, déboursé sec et devis quantitatif et estimatif (DQE) d'un bâtiment industriel 30 x 10 m, murs en agglos 15 pleins, piliers IPE 220 tous les 5 m encadrés de 2 poteaux BA, contreventements en cornières 50x50x5, entrée 6 m, toiture 2 versants à 20 %, dallage BA 20 cm double nappe HA10, semelles isolées 80 x 80 x 30 en HA12 avec tiges d'ancrage.</t>
-        </is>
-      </c>
+          <t>ENTREPRISE</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Auteur</t>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Raison sociale</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Moulo Jean Claude - Technicien Génie Civil BTP - Abidjan</t>
+          <t>ASSEYA SILVER CONSTRUCTION (ASC) - Construction métallique et bâtiment</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Siège</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>04/10/2026 - prix du marché d'Abidjan à confirmer par cotations fournisseurs</t>
+          <t>Bouaké</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="4" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Téléphone</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>07 08 39 02 66 / 05 05 10 76 82</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>COMMENT MODIFIER</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>asseyasilver@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Cellules bleues sur fond jaune</t>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>N° CC / RCCM</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Données modifiables : dimensions, épaisseurs, prix unitaires, rendements, coefficients. Tout le reste se recalcule automatiquement.</t>
+          <t>2245191 D / CI-BKE-01-2022-B13-00153</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Texte noir</t>
+          <t>Banque</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Formules - ne pas écraser.</t>
+          <t>Bank of Africa - compte n° 004619070000</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Sol de bonne portance</t>
+          <t>Régime fiscal</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Feuille « Paramètres » : mettre p_EPLAT = 0,20 (une seule couche de latérite) au lieu de 0,40.</t>
+          <t>TEE - Bouaké 1</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Changer un prix</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Feuille « Prix » colonne D : la modification se répercute sur tous les sous-détails, le DS et le DQE.</t>
-        </is>
-      </c>
+      <c r="B12" s="5" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Changer un rendement</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Objet</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Feuille « Sous-détails » colonne F (quantité par unité d'ouvrage).</t>
+          <t>Métré, déboursé sec et devis quantitatif et estimatif (DQE) d'un bâtiment industriel 30 x 10 m, murs en agglos 15 pleins, piliers IPE 220 tous les 5 m encadrés de 2 poteaux BA, contreventements en cornières 50x50x5, entrée 6 m, toiture 2 versants à 20 %, dallage BA 20 cm double nappe HA10, semelles isolées 80 x 80 x 30 en HA12 avec tiges d'ancrage.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Auteur</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Moulo Jean Claude - Technicien Génie Civil BTP - Abidjan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>FEUILLES</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr"/>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>04/10/2026 - prix du marché d'Abidjan à confirmer par cotations fournisseurs</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Paramètres</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Dimensions, hypothèses, coefficients K et TVA, grandeurs calculées (noms p_...).</t>
-        </is>
-      </c>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Prix</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Prix de base : matériaux, main-d'œuvre (h.j), matériel (noms px_...).</t>
-        </is>
-      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>COMMENT MODIFIER</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Aciers</t>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Cellules bleues sur fond jaune</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Nomenclature des aciers HA6 / HA10 / HA12 par lot, nombre de barres de 12 m.</t>
+          <t>Données modifiables : dimensions, épaisseurs, prix unitaires, rendements, coefficients. Tout le reste se recalcule automatiquement.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Métré</t>
+          <t>Texte noir</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Avant-métré : formule de chaque quantité (noms q_...).</t>
+          <t>Formules - ne pas écraser.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Sous-détails</t>
+          <t>Sol de bonne portance</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Décomposition matériaux / main-d'œuvre / matériel de chaque prix unitaire.</t>
+          <t>Feuille « Paramètres » : mettre p_EPLAT = 0,20 (une seule couche de latérite) au lieu de 0,40.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Déboursé sec</t>
+          <t>Changer un prix</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Déboursé sec par article et par lot, répartition par nature.</t>
+          <t>Feuille « Prix » colonne D : la modification se répercute sur tous les sous-détails, le DS et le DQE.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>DQE</t>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Changer un rendement</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Devis quantitatif et estimatif : PU = DS x K arrondi à 5 FCFA, récapitulatif HT / TVA 18 % / TTC.</t>
+          <t>Feuille « Sous-détails » colonne F (quantité par unité d'ouvrage).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Matériaux et MO</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Liste de commande des matériaux et besoins en main-d'œuvre et matériel.</t>
-        </is>
-      </c>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="B24" s="5" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>FEUILLES</t>
+        </is>
+      </c>
       <c r="C24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>HYPOTHÈSES CLÉS</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Paramètres</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Dimensions, hypothèses, coefficients K et TVA, grandeurs calculées (noms p_...).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Piliers</t>
+          <t>Prix</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>17 piliers en IPE 220 (S235) de ±0,00 à +6,00 sur platine 15 mm et 4 tiges d'ancrage M20 ; 2 poteaux BA 15x15 (4 HA10, cadres HA6 e = 15) de part et d'autre de chaque IPE.</t>
+          <t>Prix de base : matériaux, main-d'œuvre (h.j), matériel (noms px_...).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Contreventements</t>
+          <t>Aciers</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Cornières 50x50x5 : 4 palées verticales en croix (travées d'extrémité des long pans) et poutre au vent dans 2 travées de toiture.</t>
+          <t>Nomenclature des aciers HA6 / HA10 / HA12 par lot, nombre de barres de 12 m.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Semelles isolées</t>
+          <t>Métré</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>80 x 80 x 30 cm, fond de fouille à -1,20 m, nappe HA12 e = 15 cm dans les 2 sens, fût BA 40 x 40 (4 HA12) jusqu'à ±0,00 recevant les 4 tiges d'ancrage M20 de la platine de l'IPE.</t>
+          <t>Avant-métré : formule de chaque quantité (noms q_...).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Dallage</t>
+          <t>Sous-détails</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>20 cm, béton dosé à 350 kg/m³, double nappe HA10 e = 20 cm, chaises HA10, polyane, joints sciés maille 5 m.</t>
+          <t>Décomposition matériaux / main-d'œuvre / matériel de chaque prix unitaire.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>Déboursé sec</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Déboursé sec par article et par lot, répartition par nature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>DQE</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Devis quantitatif et estimatif : PU = DS x K arrondi à 5 FCFA, récapitulatif HT / TVA 18 % / TTC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Matériaux et MO</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Liste de commande des matériaux et besoins en main-d'œuvre et matériel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>HYPOTHÈSES CLÉS</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Piliers</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>17 piliers en IPE 220 (S235) de ±0,00 à +6,00 sur platine 15 mm et 4 tiges d'ancrage M20 ; 2 poteaux BA 15x15 (4 HA10, cadres HA6 e = 15) de part et d'autre de chaque IPE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Contreventements</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Cornières 50x50x5 : 4 palées verticales en croix (travées d'extrémité des long pans) et poutre au vent dans 2 travées de toiture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Semelles isolées</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>80 x 80 x 30 cm, fond de fouille à -1,20 m, nappe HA12 e = 15 cm dans les 2 sens, fût BA 40 x 40 (4 HA12) jusqu'à ±0,00 recevant les 4 tiges d'ancrage M20 de la platine de l'IPE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Dallage</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>20 cm, béton dosé à 350 kg/m³, double nappe HA10 e = 20 cm, chaises HA10, polyane, joints sciés maille 5 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
           <t>Forme</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Purge et rechargement en latérite par couches de 20 cm compactées à 95 % OPM : 40 cm si mauvaise portance (valeur par défaut), 20 cm sinon.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="5" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Options</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Lots 6 à 8 (enduits, fermes + pannes Z 120x2 + tôles bacs 5 ondes, portail) chiffrés séparément.</t>
         </is>
@@ -1099,13 +1262,14 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RNotice du classeur</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RNotice du classeur</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1128,14 +1292,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Paramètres et hypothèses - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Paramètres et hypothèses - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -3080,8 +3244,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RParamètres et hypothèses</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RParamètres et hypothèses</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3109,14 +3273,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prix de base - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Prix de base - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -4391,8 +4555,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RPrix de base</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RPrix de base</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -4422,14 +4586,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nomenclature des aciers - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Nomenclature des aciers - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -5292,8 +5456,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RNomenclature des aciers</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RNomenclature des aciers</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5322,14 +5486,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Avant-métré - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Avant-métré - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -6876,8 +7040,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RAvant-métré</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RAvant-métré</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6911,14 +7075,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sous-détails de prix (déboursé sec unitaire) - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Sous-détails de prix (déboursé sec unitaire) - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -21685,8 +21849,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RSous-détails de prix (déboursé sec unitaire)</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RSous-détails de prix (déboursé sec unitaire)</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -21722,14 +21886,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Déboursé sec - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Déboursé sec - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -25108,8 +25272,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RDéboursé sec</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RDéboursé sec</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -25124,7 +25288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -25139,14 +25303,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Devis quantitatif et estimatif - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Devis quantitatif et estimatif - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -27343,7 +27507,21 @@
     <row r="102">
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Fait à Abidjan, le 04/10/2026 - Moulo Jean Claude, Technicien Génie Civil BTP</t>
+          <t>Fait à Abidjan, le 04/10/2026 - Établi par Moulo Jean Claude, Technicien Génie Civil BTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Pour ASSEYA SILVER CONSTRUCTION : cachet et signature</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="41" t="inlineStr">
+        <is>
+          <t>ASSEYA SILVER CONSTRUCTION - N° CC : 2245191 D - RCCM : CI-BKE-01-2022-B13-00153 - Bank of Africa - compte n° 004619070000 - Impôts : TEE - Bouaké 1</t>
         </is>
       </c>
     </row>
@@ -27351,13 +27529,14 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RDevis quantitatif et estimatif</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RDevis quantitatif et estimatif</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -27384,14 +27563,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOULO JEAN CLAUDE - Technicien Génie Civil BTP - Abidjan, Côte d'Ivoire</t>
+          <t>ASSEYA SILVER CONSTRUCTION - Construction métallique et bâtiment - Bouaké - Tél : 07 08 39 02 66 / 05 05 10 76 82 - Email : asseyasilver@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Besoins en matériaux, main-d'œuvre et matériel - Construction d'un bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - BAEL 91 mod. 99 / EC2</t>
+          <t>Besoins en matériaux, main-d'œuvre et matériel - Bâtiment industriel 30,00 x 10,00 m - 04/10/2026 - établi par Moulo Jean Claude, Technicien Génie Civil BTP - BAEL 91 mod. 99 / EC2</t>
         </is>
       </c>
     </row>
@@ -29351,8 +29530,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LMoulo Jean Claude - Technicien Génie Civil BTP&amp;RBesoins en matériaux, main-d'œuvre et matériel</oddHeader>
-    <oddFooter>&amp;CPage &amp;P / &amp;N</oddFooter>
+    <oddHeader>&amp;LASSEYA SILVER CONSTRUCTION - établi par Moulo Jean Claude&amp;RBesoins en matériaux, main-d'œuvre et matériel</oddHeader>
+    <oddFooter>&amp;LASSEYA SILVER CONSTRUCTION - N° CC 2245191 D - RCCM CI-BKE-01-2022-B13-00153&amp;RPage &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>